<commit_message>
Archive validated agency evidence
</commit_message>
<xml_diff>
--- a/data/snapshots/ca.xlsx
+++ b/data/snapshots/ca.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jchinn2\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{29AF7EE8-79B1-4F51-BE6A-4B705A337962}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CFE79D4D-0B77-47F4-A288-FAD4FDF0655F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="751" xr2:uid="{3EA4B9A5-CE9D-4ACF-B45F-4158810915D4}"/>
   </bookViews>
@@ -15363,14 +15363,14 @@
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9CEAC05D-976A-4D1B-BF88-C07869576FC8}">
   <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <ds:schemaRef ds:uri="9ac7e9dd-8d2d-4750-b54a-f534515ac3a2"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="82b749e3-8208-459a-bfc0-9b428d09cbab"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
   </ds:schemaRefs>

</xml_diff>